<commit_message>
App v2: piezas, camiones por ciclos, personal entero y trabajadores enumerados, tiempo real y contingencia
- Pedidos de piezas individuales por tipo (VE/COMB), sin ensamblaje
- Expediciones cada 1,5 h (16 ciclos/día) con los camiones de 15 m² necesarios
- El stock de seguridad puede consumirse por expedición y se repone con prioridad máxima
- Franja solar 11-14 h; la célula 10 no puede pararse ni averiarse
- Entrada manual: bajas por turno (todos los roles), paradas (programadas/avería) y demanda
- Personal entero por hora y plantilla por turno; trabajadores enumerados asignados puesto a puesto
- Pestañas Planta en tiempo real, Trabajadores y Contingencia; recálculo automático
- Corregido el stock desfasado en incidencias encadenadas
- Definición del plan manual; demo con 1.500 coches/día (2:1 combustión:VE)
</commit_message>
<xml_diff>
--- a/Claude code/kwd_motor/data/entrada_ejemplo.xlsx
+++ b/Claude code/kwd_motor/data/entrada_ejemplo.xlsx
@@ -14,9 +14,9 @@
     <sheet name="DemandaSemanal" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="CorreccionDiaria" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="StockActual" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Disponibilidad" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Mantenimientos" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="RecursosReales" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Bajas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="BajasTrabajadores" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Paradas" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Expediciones" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,11 +481,6 @@
           <t>kw</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>piezas_por_conjunto</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -520,9 +515,6 @@
       <c r="J2" t="n">
         <v>22</v>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -557,9 +549,6 @@
       <c r="J3" t="n">
         <v>22</v>
       </c>
-      <c r="K3" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -594,9 +583,6 @@
       <c r="J4" t="n">
         <v>115.42</v>
       </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -631,9 +617,6 @@
       <c r="J5" t="n">
         <v>45.1</v>
       </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -668,9 +651,6 @@
       <c r="J6" t="n">
         <v>10</v>
       </c>
-      <c r="K6" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -705,9 +685,6 @@
       <c r="J7" t="n">
         <v>15</v>
       </c>
-      <c r="K7" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -742,9 +719,6 @@
       <c r="J8" t="n">
         <v>16</v>
       </c>
-      <c r="K8" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -779,9 +753,6 @@
       <c r="J9" t="n">
         <v>13.79</v>
       </c>
-      <c r="K9" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -816,9 +787,6 @@
       <c r="J10" t="n">
         <v>10.46</v>
       </c>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -853,9 +821,6 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -890,9 +855,6 @@
       <c r="J12" t="n">
         <v>51</v>
       </c>
-      <c r="K12" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -927,9 +889,6 @@
       <c r="J13" t="n">
         <v>51</v>
       </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -964,9 +923,6 @@
       <c r="J14" t="n">
         <v>79.59999999999999</v>
       </c>
-      <c r="K14" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1001,9 +957,6 @@
       <c r="J15" t="n">
         <v>77.94</v>
       </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1038,9 +991,6 @@
       <c r="J16" t="n">
         <v>77.95</v>
       </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1074,9 +1024,6 @@
       </c>
       <c r="J17" t="n">
         <v>25</v>
-      </c>
-      <c r="K17" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1090,62 +1037,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>fecha</t>
+          <t>celula</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>turno</t>
+          <t>desde</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>operarios</t>
+          <t>hasta</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>picking</t>
+          <t>tipo</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>carretilleros</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>mto</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>calidad</t>
+          <t>tecnicos</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46297</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="A2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46297.58333333334</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>46297.91666666666</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PROGRAMADA</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1169,12 +1108,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>chasis_ve</t>
+          <t>piezas_ve</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>chasis_comb</t>
+          <t>piezas_comb</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1444,15 +1383,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>camiones_dia</t>
+          <t>ciclos_dia</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Camiones por día laborable (F6)</t>
+          <t>Ciclos de expedición por día laborable (F6)</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1406,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Intervalo entre camiones, horas (F6)</t>
+          <t>Intervalo entre ciclos de expedición, horas (F6)</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1421,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hora del primer camión del día (F6)</t>
+          <t>Hora del primer ciclo del día (F6)</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1436,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>m² máximos liberados por camión (F6)</t>
+          <t>m² máximos por camión (F6)</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1462,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1643,11 +1582,11 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tiempo límite del solver por plan, segundos</t>
+          <t>Tiempo límite total del solver por plan (2 fases), segundos</t>
         </is>
       </c>
     </row>
@@ -1693,6 +1632,21 @@
       <c r="C22" t="inlineStr">
         <is>
           <t>Gap relativo MIP aceptado por el solver (la spec pide 0; relajado por velocidad)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>penalizacion_ss</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>50</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Penalización de prioridad máxima por unidad normalizada (s/SS) y hora de stock de seguridad consumido (F20)</t>
         </is>
       </c>
     </row>
@@ -1718,12 +1672,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>chasis_ve</t>
+          <t>piezas_ve</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>chasis_comb</t>
+          <t>piezas_comb</t>
         </is>
       </c>
     </row>
@@ -1732,10 +1686,10 @@
         <v>46293</v>
       </c>
       <c r="B2" t="n">
-        <v>2400</v>
+        <v>2500</v>
       </c>
       <c r="C2" t="n">
-        <v>1600</v>
+        <v>5000</v>
       </c>
     </row>
   </sheetData>
@@ -1760,12 +1714,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>chasis_ve</t>
+          <t>piezas_ve</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>chasis_comb</t>
+          <t>piezas_comb</t>
         </is>
       </c>
     </row>
@@ -1777,7 +1731,7 @@
         <v>520</v>
       </c>
       <c r="C2" t="n">
-        <v>300</v>
+        <v>980</v>
       </c>
     </row>
   </sheetData>
@@ -1811,7 +1765,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
     <row r="3">
@@ -1819,7 +1773,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4">
@@ -1827,7 +1781,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="5">
@@ -1835,7 +1789,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="6">
@@ -1843,7 +1797,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7">
@@ -1851,7 +1805,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8">
@@ -1859,7 +1813,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9">
@@ -1867,7 +1821,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="10">
@@ -1875,7 +1829,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="11">
@@ -1883,7 +1837,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12">
@@ -1891,7 +1845,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13">
@@ -1899,7 +1853,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="n">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="14">
@@ -1907,7 +1861,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="n">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="15">
@@ -1915,7 +1869,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="n">
-        <v>720</v>
+        <v>800</v>
       </c>
     </row>
     <row r="16">
@@ -1923,7 +1877,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -1937,29 +1891,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>celula</t>
+          <t>fecha</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>estado</t>
+          <t>turno</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>desde</t>
+          <t>operarios</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>hasta</t>
-        </is>
+          <t>picking</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>carretilleros</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>mto</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>calidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1973,7 +1967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1984,34 +1978,8 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>turno</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>celula</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>tecnicos</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46297</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>13</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
+          <t>trabajador</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>